<commit_message>
Add TabDDPM backend, multi-GPU runners, and refresh HPO Excel reports.
Complete TabDDPM on all 15 datasets, include it in Adult-style workbooks, and add shared report/parallel-GPU tooling.
</commit_message>
<xml_diff>
--- a/results/classification/3_adult/adult_HPO_results.xlsx
+++ b/results/classification/3_adult/adult_HPO_results.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Performance Metrics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Hyperparameters" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Metric Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Performance Metrics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Best Hyperparameters" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
@@ -44,8 +50,23 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -64,27 +85,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="005B9BD5"/>
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0070AD47"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ED7D31"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="007F7F7F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00833C0C"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -93,7 +104,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -107,51 +118,96 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -542,34 +598,34 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Objective = 0.4 × Fidelity  +  0.4 × Utility (Accuracy)  −  0.2 × Privacy Risk</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>COLOR / ROLE</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>In Objective?</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -581,211 +637,211 @@
           <t>OBJECTIVE</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Final scalar score used for ranking</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>YES — result</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Sort generators by this</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>MAIN — Fidelity</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Statistical similarity</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>+0.4</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Higher better</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>MAIN — Utility (Accuracy)</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>ML usefulness via Accuracy</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>+0.4</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Higher better</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>MAIN — Privacy Risk</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Leakage / memorization risk</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>−0.2</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Higher worse (subtracted)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>SUB → Fidelity</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>KS Similarity, Corr Similarity</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>Support / explain Fidelity</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>SUB → Utility</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>TSTR/TRTR Acc, Gap, per-classifier</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>Support / explain Utility</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>SUB → Privacy</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>MIA AUC, NNDR, DCR</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Support / explain Privacy Risk</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>REFERENCE ONLY</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>F1 metrics &amp; original Optuna F1-HPO</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Not used in current Objective</t>
         </is>
@@ -799,432 +855,432 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Definition</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>In Objective?</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>How it enters</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>OBJECTIVE</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Objective</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>0.4·Fidelity + 0.4·Utility(Accuracy) − 0.2·PrivacyRisk</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Final ranking score</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Fidelity</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="13" t="inlineStr">
         <is>
           <t>avg(KS Similarity, Corr Similarity)</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>YES (+0.4)</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>Main component</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>SUB → Fidelity</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>KS Similarity</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="13" t="inlineStr">
         <is>
           <t>1 − KS distance, averaged over columns</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="13" t="inlineStr">
         <is>
           <t>Builds Fidelity</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>SUB → Fidelity</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Corr Similarity</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>Correlation matrix similarity real vs synthetic</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="13" t="inlineStr">
         <is>
           <t>Builds Fidelity</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Utility (Accuracy)</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="13" t="inlineStr">
         <is>
           <t>1 − clip(max(TRTR_Acc − TSTR_Acc, 0), 0, 1)</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>YES (+0.4)</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="13" t="inlineStr">
         <is>
           <t>Main component</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>SUB → Utility</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>TSTR Accuracy</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t>Train on Synthetic, Test on Real (mean of 3 clfs)</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="13" t="inlineStr">
         <is>
           <t>Builds Utility</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>SUB → Utility</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>TRTR Accuracy</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
         <is>
           <t>Train on Real, Test on Real baseline</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="13" t="inlineStr">
         <is>
           <t>Builds Utility</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>SUB → Utility</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>Accuracy Gap</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="13" t="inlineStr">
         <is>
           <t>TRTR Accuracy − TSTR Accuracy</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="13" t="inlineStr">
         <is>
           <t>Builds Utility</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>SUB → Utility</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>TSTR/TRTR Acc per clf</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>LogReg, RF, Decision Tree</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E27" s="13" t="inlineStr">
         <is>
           <t>Builds Utility</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Privacy Risk</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="13" t="inlineStr">
         <is>
           <t>0.5·MIA_AUC + 0.3·NNDR_norm + 0.2·DCR_norm</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>YES (−0.2)</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="13" t="inlineStr">
         <is>
           <t>Main component (subtracted)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>SUB → Privacy</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>MIA AUC</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="13" t="inlineStr">
         <is>
           <t>Membership inference attack AUC</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E29" s="13" t="inlineStr">
         <is>
           <t>Builds Privacy Risk</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>SUB → Privacy</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>NNDR</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="13" t="inlineStr">
         <is>
           <t>Nearest-neighbor distance ratio</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="13" t="inlineStr">
         <is>
           <t>Builds Privacy Risk</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>SUB → Privacy</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="13" t="inlineStr">
         <is>
           <t>DCR</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="13" t="inlineStr">
         <is>
           <t>Distance to closest record</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" s="13" t="inlineStr">
         <is>
           <t>Builds Privacy Risk</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>Utility (F1) / TSTR F1 / TRTR F1 / F1 Gap</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>F1-based utility used during Optuna HPO</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="14" t="inlineStr">
         <is>
           <t>Reference only</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>REFERENCE</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>Objective (F1 HPO)</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="14" t="inlineStr">
         <is>
           <t>Score Optuna maximized during search</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" s="14" t="inlineStr">
         <is>
           <t>Reference only</t>
         </is>
@@ -1238,17 +1294,22 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Adult treated as COMPLETE with 6 generators: GaussianCopula, CopulaGAN, CTGAN, TVAE, CTAB-GAN+, WGAN-GP. ForestDiffusion skipped (incomplete / excluded). TabDDPM unavailable. Sampling: max 1000 rows, balanced classes, seed 42. Train=800, Test=200. Report date: 2026-08-26.</t>
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>Adult Census HPO report. Generators: GaussianCopula, CopulaGAN, CTGAN, TVAE, CTAB-GAN+, WGAN-GP, TabDDPM. All 7 generators complete. Sampling: max 1000 rows, seed 42. Train=800, Test=200. Utility models: Logistic Regression, Random Forest, Decision Tree. Report date: 2026-09-28.</t>
         </is>
       </c>
     </row>
     <row r="38"/>
     <row r="39"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="6">
+    <mergeCell ref="A4:E4"/>
     <mergeCell ref="A37:E39"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1260,760 +1321,851 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="12" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="6" t="n"/>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>OBJECTIVE</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>MAIN METRICS (used in Objective)</t>
         </is>
       </c>
-      <c r="E1" s="7" t="n"/>
-      <c r="F1" s="7" t="n"/>
+      <c r="E1" s="17" t="n"/>
+      <c r="F1" s="18" t="n"/>
       <c r="G1" s="8" t="inlineStr">
         <is>
           <t>SUB → Fidelity</t>
         </is>
       </c>
-      <c r="H1" s="8" t="n"/>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="H1" s="19" t="n"/>
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>SUB → Utility (Accuracy)</t>
         </is>
       </c>
-      <c r="J1" s="9" t="n"/>
-      <c r="K1" s="9" t="n"/>
-      <c r="L1" s="9" t="n"/>
-      <c r="M1" s="9" t="n"/>
-      <c r="N1" s="9" t="n"/>
-      <c r="O1" s="9" t="n"/>
-      <c r="P1" s="9" t="n"/>
-      <c r="Q1" s="9" t="n"/>
-      <c r="R1" s="10" t="inlineStr">
+      <c r="J1" s="20" t="n"/>
+      <c r="K1" s="20" t="n"/>
+      <c r="L1" s="20" t="n"/>
+      <c r="M1" s="20" t="n"/>
+      <c r="N1" s="20" t="n"/>
+      <c r="O1" s="20" t="n"/>
+      <c r="P1" s="20" t="n"/>
+      <c r="Q1" s="19" t="n"/>
+      <c r="R1" s="8" t="inlineStr">
         <is>
           <t>SUB → Privacy Risk</t>
         </is>
       </c>
-      <c r="S1" s="10" t="n"/>
-      <c r="T1" s="10" t="n"/>
-      <c r="U1" s="11" t="inlineStr">
+      <c r="S1" s="20" t="n"/>
+      <c r="T1" s="19" t="n"/>
+      <c r="U1" s="10" t="inlineStr">
         <is>
           <t>REFERENCE ONLY (NOT in Objective)</t>
         </is>
       </c>
-      <c r="V1" s="11" t="n"/>
-      <c r="W1" s="11" t="n"/>
-      <c r="X1" s="11" t="n"/>
-      <c r="Y1" s="11" t="n"/>
-      <c r="Z1" s="12" t="inlineStr">
+      <c r="V1" s="21" t="n"/>
+      <c r="W1" s="21" t="n"/>
+      <c r="X1" s="21" t="n"/>
+      <c r="Y1" s="22" t="n"/>
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>Run</t>
         </is>
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Generator</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Objective
 0.4F+0.4U−0.2P</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Fidelity
 (+0.4)</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Utility (Accuracy)
 (+0.4)</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Privacy Risk
 (−0.2)</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>KS Similarity</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Corr Similarity</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>TSTR Accuracy</t>
         </is>
       </c>
-      <c r="J2" s="9" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>TRTR Accuracy</t>
         </is>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Accuracy Gap</t>
         </is>
       </c>
-      <c r="L2" s="9" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>TSTR Acc (LogReg)</t>
         </is>
       </c>
-      <c r="M2" s="9" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>TSTR Acc (RF)</t>
         </is>
       </c>
-      <c r="N2" s="9" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>TSTR Acc (DT)</t>
         </is>
       </c>
-      <c r="O2" s="9" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>TRTR Acc (LogReg)</t>
         </is>
       </c>
-      <c r="P2" s="9" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>TRTR Acc (RF)</t>
         </is>
       </c>
-      <c r="Q2" s="9" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>TRTR Acc (DT)</t>
         </is>
       </c>
-      <c r="R2" s="10" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>MIA AUC</t>
         </is>
       </c>
-      <c r="S2" s="10" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>NNDR</t>
         </is>
       </c>
-      <c r="T2" s="10" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>DCR</t>
         </is>
       </c>
-      <c r="U2" s="11" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>Utility (F1)</t>
         </is>
       </c>
-      <c r="V2" s="11" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>TSTR F1</t>
         </is>
       </c>
-      <c r="W2" s="11" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>TRTR F1</t>
         </is>
       </c>
-      <c r="X2" s="11" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>F1 Gap</t>
         </is>
       </c>
-      <c r="Y2" s="11" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>Objective (F1 HPO)</t>
         </is>
       </c>
-      <c r="Z2" s="12" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>Time (s)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="n">
+      <c r="A3" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>CopulaGAN</t>
         </is>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="23" t="n">
         <v>0.6254999999999999</v>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="23" t="n">
         <v>0.9172</v>
       </c>
-      <c r="E3" s="13" t="n">
+      <c r="E3" s="23" t="n">
         <v>0.9467</v>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="F3" s="23" t="n">
         <v>0.6002</v>
       </c>
-      <c r="G3" s="13" t="n">
+      <c r="G3" s="23" t="n">
         <v>0.9012</v>
       </c>
-      <c r="H3" s="13" t="n">
+      <c r="H3" s="23" t="n">
         <v>0.9331</v>
       </c>
-      <c r="I3" s="13" t="n">
+      <c r="I3" s="23" t="n">
         <v>0.785</v>
       </c>
-      <c r="J3" s="13" t="n">
+      <c r="J3" s="23" t="n">
         <v>0.8383</v>
       </c>
-      <c r="K3" s="13" t="n">
+      <c r="K3" s="23" t="n">
         <v>0.0533</v>
       </c>
-      <c r="L3" s="13" t="n">
+      <c r="L3" s="23" t="n">
         <v>0.795</v>
       </c>
-      <c r="M3" s="13" t="n">
+      <c r="M3" s="23" t="n">
         <v>0.805</v>
       </c>
-      <c r="N3" s="13" t="n">
+      <c r="N3" s="23" t="n">
         <v>0.755</v>
       </c>
-      <c r="O3" s="13" t="n">
+      <c r="O3" s="23" t="n">
         <v>0.83</v>
       </c>
-      <c r="P3" s="13" t="n">
+      <c r="P3" s="23" t="n">
         <v>0.86</v>
       </c>
-      <c r="Q3" s="13" t="n">
+      <c r="Q3" s="23" t="n">
         <v>0.825</v>
       </c>
-      <c r="R3" s="13" t="n">
+      <c r="R3" s="23" t="n">
         <v>0.7718</v>
       </c>
-      <c r="S3" s="13" t="n">
+      <c r="S3" s="23" t="n">
         <v>0.9522</v>
       </c>
-      <c r="T3" s="13" t="n">
+      <c r="T3" s="23" t="n">
         <v>2.1707</v>
       </c>
-      <c r="U3" s="13" t="n">
+      <c r="U3" s="23" t="n">
         <v>0.9359</v>
       </c>
-      <c r="V3" s="13" t="n">
+      <c r="V3" s="23" t="n">
         <v>0.7737000000000001</v>
       </c>
-      <c r="W3" s="13" t="n">
+      <c r="W3" s="23" t="n">
         <v>0.8378</v>
       </c>
-      <c r="X3" s="13" t="n">
+      <c r="X3" s="23" t="n">
         <v>0.0641</v>
       </c>
-      <c r="Y3" s="13" t="n">
-        <v>0.6212</v>
-      </c>
-      <c r="Z3" s="13" t="n">
+      <c r="Y3" s="23" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="Z3" s="23" t="n">
         <v>1249.6</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="n">
+      <c r="A4" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>TVAE</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
+      <c r="C4" s="24" t="n">
         <v>0.6138</v>
       </c>
-      <c r="D4" s="14" t="n">
+      <c r="D4" s="24" t="n">
         <v>0.9127</v>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="E4" s="24" t="n">
         <v>0.95</v>
       </c>
-      <c r="F4" s="14" t="n">
+      <c r="F4" s="24" t="n">
         <v>0.6562</v>
       </c>
-      <c r="G4" s="14" t="n">
+      <c r="G4" s="24" t="n">
         <v>0.8764</v>
       </c>
-      <c r="H4" s="14" t="n">
+      <c r="H4" s="24" t="n">
         <v>0.9489</v>
       </c>
-      <c r="I4" s="14" t="n">
+      <c r="I4" s="24" t="n">
         <v>0.7883</v>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="24" t="n">
         <v>0.8383</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="K4" s="24" t="n">
         <v>0.05</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="L4" s="24" t="n">
         <v>0.8</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="M4" s="24" t="n">
         <v>0.8</v>
       </c>
-      <c r="N4" s="14" t="n">
+      <c r="N4" s="24" t="n">
         <v>0.765</v>
       </c>
-      <c r="O4" s="14" t="n">
+      <c r="O4" s="24" t="n">
         <v>0.83</v>
       </c>
-      <c r="P4" s="14" t="n">
+      <c r="P4" s="24" t="n">
         <v>0.86</v>
       </c>
-      <c r="Q4" s="14" t="n">
+      <c r="Q4" s="24" t="n">
         <v>0.825</v>
       </c>
-      <c r="R4" s="14" t="n">
+      <c r="R4" s="24" t="n">
         <v>0.8558</v>
       </c>
-      <c r="S4" s="14" t="n">
+      <c r="S4" s="24" t="n">
         <v>0.9056999999999999</v>
       </c>
-      <c r="T4" s="14" t="n">
+      <c r="T4" s="24" t="n">
         <v>1.5677</v>
       </c>
-      <c r="U4" s="14" t="n">
+      <c r="U4" s="24" t="n">
         <v>0.9360000000000001</v>
       </c>
-      <c r="V4" s="14" t="n">
+      <c r="V4" s="24" t="n">
         <v>0.7738</v>
       </c>
-      <c r="W4" s="14" t="n">
+      <c r="W4" s="24" t="n">
         <v>0.8378</v>
       </c>
-      <c r="X4" s="14" t="n">
+      <c r="X4" s="24" t="n">
         <v>0.064</v>
       </c>
-      <c r="Y4" s="14" t="n">
-        <v>0.6082</v>
-      </c>
-      <c r="Z4" s="14" t="n">
+      <c r="Y4" s="24" t="n">
+        <v>0.6322</v>
+      </c>
+      <c r="Z4" s="24" t="n">
         <v>417.4</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="n">
+      <c r="A5" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>CTGAN</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" s="24" t="n">
         <v>0.5869</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="24" t="n">
         <v>0.8877</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="24" t="n">
         <v>0.9133</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="24" t="n">
         <v>0.6677</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="24" t="n">
         <v>0.8218</v>
       </c>
-      <c r="H5" s="14" t="n">
+      <c r="H5" s="24" t="n">
         <v>0.9537</v>
       </c>
-      <c r="I5" s="14" t="n">
+      <c r="I5" s="24" t="n">
         <v>0.7517</v>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="24" t="n">
         <v>0.8383</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="K5" s="24" t="n">
         <v>0.0867</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="L5" s="24" t="n">
         <v>0.79</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="M5" s="24" t="n">
         <v>0.79</v>
       </c>
-      <c r="N5" s="14" t="n">
+      <c r="N5" s="24" t="n">
         <v>0.675</v>
       </c>
-      <c r="O5" s="14" t="n">
+      <c r="O5" s="24" t="n">
         <v>0.83</v>
       </c>
-      <c r="P5" s="14" t="n">
+      <c r="P5" s="24" t="n">
         <v>0.86</v>
       </c>
-      <c r="Q5" s="14" t="n">
+      <c r="Q5" s="24" t="n">
         <v>0.825</v>
       </c>
-      <c r="R5" s="14" t="n">
+      <c r="R5" s="24" t="n">
         <v>0.9004</v>
       </c>
-      <c r="S5" s="14" t="n">
+      <c r="S5" s="24" t="n">
         <v>0.9417</v>
       </c>
-      <c r="T5" s="14" t="n">
+      <c r="T5" s="24" t="n">
         <v>2.0975</v>
       </c>
-      <c r="U5" s="14" t="n">
+      <c r="U5" s="24" t="n">
         <v>0.8848</v>
       </c>
-      <c r="V5" s="14" t="n">
+      <c r="V5" s="24" t="n">
         <v>0.7226</v>
       </c>
-      <c r="W5" s="14" t="n">
+      <c r="W5" s="24" t="n">
         <v>0.8378</v>
       </c>
-      <c r="X5" s="14" t="n">
+      <c r="X5" s="24" t="n">
         <v>0.1152</v>
       </c>
-      <c r="Y5" s="14" t="n">
-        <v>0.5755</v>
-      </c>
-      <c r="Z5" s="14" t="n">
+      <c r="Y5" s="24" t="n">
+        <v>0.6089</v>
+      </c>
+      <c r="Z5" s="24" t="n">
         <v>2697.7</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="n">
+      <c r="A6" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>GaussianCopula</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="24" t="n">
         <v>0.5667</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="24" t="n">
         <v>0.8414</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="24" t="n">
         <v>0.9317</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="24" t="n">
         <v>0.7124</v>
       </c>
-      <c r="G6" s="14" t="n">
+      <c r="G6" s="24" t="n">
         <v>0.7338</v>
       </c>
-      <c r="H6" s="14" t="n">
+      <c r="H6" s="24" t="n">
         <v>0.949</v>
       </c>
-      <c r="I6" s="14" t="n">
+      <c r="I6" s="24" t="n">
         <v>0.77</v>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="24" t="n">
         <v>0.8383</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="K6" s="24" t="n">
         <v>0.0683</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="L6" s="24" t="n">
         <v>0.76</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="M6" s="24" t="n">
         <v>0.8</v>
       </c>
-      <c r="N6" s="14" t="n">
+      <c r="N6" s="24" t="n">
         <v>0.75</v>
       </c>
-      <c r="O6" s="14" t="n">
+      <c r="O6" s="24" t="n">
         <v>0.83</v>
       </c>
-      <c r="P6" s="14" t="n">
+      <c r="P6" s="24" t="n">
         <v>0.86</v>
       </c>
-      <c r="Q6" s="14" t="n">
+      <c r="Q6" s="24" t="n">
         <v>0.825</v>
       </c>
-      <c r="R6" s="14" t="n">
+      <c r="R6" s="24" t="n">
         <v>0.999</v>
       </c>
-      <c r="S6" s="14" t="n">
+      <c r="S6" s="24" t="n">
         <v>0.9569</v>
       </c>
-      <c r="T6" s="14" t="n">
+      <c r="T6" s="24" t="n">
         <v>2.39</v>
       </c>
-      <c r="U6" s="14" t="n">
+      <c r="U6" s="24" t="n">
         <v>0.9249000000000001</v>
       </c>
-      <c r="V6" s="14" t="n">
+      <c r="V6" s="24" t="n">
         <v>0.7627</v>
       </c>
-      <c r="W6" s="14" t="n">
+      <c r="W6" s="24" t="n">
         <v>0.8378</v>
       </c>
-      <c r="X6" s="14" t="n">
+      <c r="X6" s="24" t="n">
         <v>0.0751</v>
       </c>
-      <c r="Y6" s="14" t="n">
+      <c r="Y6" s="24" t="n">
         <v>0.5639999999999999</v>
       </c>
-      <c r="Z6" s="14" t="n">
+      <c r="Z6" s="24" t="n">
         <v>24.7</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n">
+      <c r="A7" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>WGAN-GP</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="24" t="n">
         <v>0.5432</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="24" t="n">
         <v>0.8786</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="24" t="n">
         <v>0.8383</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="24" t="n">
         <v>0.7176</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="24" t="n">
         <v>0.7986</v>
       </c>
-      <c r="H7" s="14" t="n">
+      <c r="H7" s="24" t="n">
         <v>0.9586</v>
       </c>
-      <c r="I7" s="14" t="n">
+      <c r="I7" s="24" t="n">
         <v>0.6767</v>
       </c>
-      <c r="J7" s="14" t="n">
+      <c r="J7" s="24" t="n">
         <v>0.8383</v>
       </c>
-      <c r="K7" s="14" t="n">
+      <c r="K7" s="24" t="n">
         <v>0.1617</v>
       </c>
-      <c r="L7" s="14" t="n">
+      <c r="L7" s="24" t="n">
         <v>0.73</v>
       </c>
-      <c r="M7" s="14" t="n">
+      <c r="M7" s="24" t="n">
         <v>0.705</v>
       </c>
-      <c r="N7" s="14" t="n">
+      <c r="N7" s="24" t="n">
         <v>0.595</v>
       </c>
-      <c r="O7" s="14" t="n">
+      <c r="O7" s="24" t="n">
         <v>0.83</v>
       </c>
-      <c r="P7" s="14" t="n">
+      <c r="P7" s="24" t="n">
         <v>0.86</v>
       </c>
-      <c r="Q7" s="14" t="n">
+      <c r="Q7" s="24" t="n">
         <v>0.825</v>
       </c>
-      <c r="R7" s="14" t="n">
+      <c r="R7" s="24" t="n">
         <v>0.9999</v>
       </c>
-      <c r="S7" s="14" t="n">
+      <c r="S7" s="24" t="n">
         <v>0.9412</v>
       </c>
-      <c r="T7" s="14" t="n">
+      <c r="T7" s="24" t="n">
         <v>2.041</v>
       </c>
-      <c r="U7" s="14" t="n">
+      <c r="U7" s="24" t="n">
         <v>0.7788</v>
       </c>
-      <c r="V7" s="14" t="n">
+      <c r="V7" s="24" t="n">
         <v>0.6166</v>
       </c>
-      <c r="W7" s="14" t="n">
+      <c r="W7" s="24" t="n">
         <v>0.8378</v>
       </c>
-      <c r="X7" s="14" t="n">
+      <c r="X7" s="24" t="n">
         <v>0.2212</v>
       </c>
-      <c r="Y7" s="14" t="n">
-        <v>0.5194</v>
-      </c>
-      <c r="Z7" s="14" t="n">
+      <c r="Y7" s="24" t="n">
+        <v>0.5737</v>
+      </c>
+      <c r="Z7" s="24" t="n">
         <v>491.5</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="n">
+      <c r="A8" s="24" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>CTAB-GAN+</t>
         </is>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="24" t="n">
         <v>0.4998</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="24" t="n">
         <v>0.7148</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="24" t="n">
         <v>0.895</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="24" t="n">
         <v>0.7207</v>
       </c>
-      <c r="G8" s="14" t="n">
+      <c r="G8" s="24" t="n">
         <v>0.5158</v>
       </c>
-      <c r="H8" s="14" t="n">
+      <c r="H8" s="24" t="n">
         <v>0.9139</v>
       </c>
-      <c r="I8" s="14" t="n">
+      <c r="I8" s="24" t="n">
         <v>0.7333</v>
       </c>
-      <c r="J8" s="14" t="n">
+      <c r="J8" s="24" t="n">
         <v>0.8383</v>
       </c>
-      <c r="K8" s="14" t="n">
+      <c r="K8" s="24" t="n">
         <v>0.105</v>
       </c>
-      <c r="L8" s="14" t="n">
+      <c r="L8" s="24" t="n">
         <v>0.75</v>
       </c>
-      <c r="M8" s="14" t="n">
+      <c r="M8" s="24" t="n">
         <v>0.73</v>
       </c>
-      <c r="N8" s="14" t="n">
+      <c r="N8" s="24" t="n">
         <v>0.72</v>
       </c>
-      <c r="O8" s="14" t="n">
+      <c r="O8" s="24" t="n">
         <v>0.83</v>
       </c>
-      <c r="P8" s="14" t="n">
+      <c r="P8" s="24" t="n">
         <v>0.86</v>
       </c>
-      <c r="Q8" s="14" t="n">
+      <c r="Q8" s="24" t="n">
         <v>0.825</v>
       </c>
-      <c r="R8" s="14" t="n">
+      <c r="R8" s="24" t="n">
         <v>0.9999</v>
       </c>
-      <c r="S8" s="14" t="n">
+      <c r="S8" s="24" t="n">
         <v>0.9306</v>
       </c>
-      <c r="T8" s="14" t="n">
+      <c r="T8" s="24" t="n">
         <v>2.3749</v>
       </c>
-      <c r="U8" s="14" t="n">
+      <c r="U8" s="24" t="n">
         <v>0.8895</v>
       </c>
-      <c r="V8" s="14" t="n">
+      <c r="V8" s="24" t="n">
         <v>0.7272999999999999</v>
       </c>
-      <c r="W8" s="14" t="n">
+      <c r="W8" s="24" t="n">
         <v>0.8378</v>
       </c>
-      <c r="X8" s="14" t="n">
+      <c r="X8" s="24" t="n">
         <v>0.1105</v>
       </c>
-      <c r="Y8" s="14" t="n">
-        <v>0.4976</v>
-      </c>
-      <c r="Z8" s="14" t="n">
+      <c r="Y8" s="24" t="n">
+        <v>0.5233</v>
+      </c>
+      <c r="Z8" s="24" t="n">
         <v>2470.3</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>TabDDPM</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>0.4584</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>0.7481</v>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>0.7533</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>0.711</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>0.5894</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <v>0.9068000000000001</v>
+      </c>
+      <c r="I9" s="24" t="n">
+        <v>0.5167</v>
+      </c>
+      <c r="J9" s="24" t="n">
+        <v>0.7633</v>
+      </c>
+      <c r="K9" s="24" t="n">
+        <v>0.2467</v>
+      </c>
+      <c r="L9" s="24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M9" s="24" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="N9" s="24" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="O9" s="24" t="n">
+        <v>0.725</v>
+      </c>
+      <c r="P9" s="24" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="Q9" s="24" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="R9" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="24" t="n">
+        <v>0.9631999999999999</v>
+      </c>
+      <c r="T9" s="24" t="n">
+        <v>7.7441</v>
+      </c>
+      <c r="U9" s="24" t="n">
+        <v>0.8687</v>
+      </c>
+      <c r="V9" s="24" t="n">
+        <v>0.6447000000000001</v>
+      </c>
+      <c r="W9" s="24" t="n">
+        <v>0.776</v>
+      </c>
+      <c r="X9" s="24" t="n">
+        <v>0.1313</v>
+      </c>
+      <c r="Y9" s="24" t="n">
+        <v>0.5044999999999999</v>
+      </c>
+      <c r="Z9" s="24" t="n">
+        <v>1151.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>Color key:</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>OBJECTIVE</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>MAIN (in formula)</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>SUB-METRIC</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>REFERENCE only</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Utility(Accuracy)=1−clip(max(TRTR_Acc−TSTR_Acc,0),0,1). Adult complete with 6 generators (ForestDiffusion skipped). See Metric Guide.</t>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>Utility(Accuracy)=1−clip(max(TRTR_Acc−TSTR_Acc,0),0,1). Adult Census report with 7 generators. See Metric Guide.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="I1:Q1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A12:Z12"/>
+    <mergeCell ref="U1:Y1"/>
+    <mergeCell ref="R1:T1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2024,7 +2176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:AF8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2051,403 +2203,561 @@
     <col width="16" customWidth="1" min="22" max="22"/>
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="16" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Generator</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>epochs</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>batch_size</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>generator_lr</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>discriminator_lr</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>generator_dim</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>discriminator_dim</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>discriminator_steps</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>pac</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>default_distribution</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>embedding_dim</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>compress_dims</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>decompress_dims</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>l2scale</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>loss_factor</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>enforce_min_max_values</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>latent_dim</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>hidden_dim</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>lr</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>n_critic</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>lambda_gp</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>random_dim</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>num_channels</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>class_dim</t>
         </is>
       </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
+          <t>num_timesteps</t>
+        </is>
+      </c>
+      <c r="Z1" s="4" t="inlineStr">
+        <is>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="AA1" s="4" t="inlineStr">
+        <is>
+          <t>n_layers</t>
+        </is>
+      </c>
+      <c r="AB1" s="4" t="inlineStr">
+        <is>
+          <t>d_layers</t>
+        </is>
+      </c>
+      <c r="AC1" s="4" t="inlineStr">
+        <is>
+          <t>sample_proportion</t>
+        </is>
+      </c>
+      <c r="AD1" s="4" t="inlineStr">
+        <is>
+          <t>dropout</t>
+        </is>
+      </c>
+      <c r="AE1" s="4" t="inlineStr">
+        <is>
+          <t>scheduler</t>
+        </is>
+      </c>
+      <c r="AF1" s="4" t="inlineStr">
+        <is>
+          <t>gaussian_loss_type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>CopulaGAN</t>
         </is>
       </c>
-      <c r="B2" s="19" t="n">
+      <c r="B2" s="28" t="n">
         <v>700</v>
       </c>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="28" t="n">
         <v>200</v>
       </c>
-      <c r="D2" s="19" t="n">
+      <c r="D2" s="28" t="n">
         <v>0.0002368657480645031</v>
       </c>
-      <c r="E2" s="19" t="n">
+      <c r="E2" s="28" t="n">
         <v>0.0005222714805518795</v>
       </c>
-      <c r="F2" s="19" t="inlineStr">
+      <c r="F2" s="28" t="inlineStr">
         <is>
           <t>[128, 128]</t>
         </is>
       </c>
-      <c r="G2" s="19" t="inlineStr">
+      <c r="G2" s="28" t="inlineStr">
         <is>
           <t>[128, 128]</t>
         </is>
       </c>
-      <c r="H2" s="19" t="n">
+      <c r="H2" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="19" t="n">
+      <c r="I2" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="J2" s="19" t="inlineStr">
+      <c r="J2" s="28" t="inlineStr">
         <is>
           <t>gamma</t>
         </is>
       </c>
-      <c r="K2" s="19" t="n"/>
-      <c r="L2" s="19" t="n"/>
-      <c r="M2" s="19" t="n"/>
-      <c r="N2" s="19" t="n"/>
-      <c r="O2" s="19" t="n"/>
-      <c r="P2" s="19" t="n"/>
-      <c r="Q2" s="19" t="n"/>
-      <c r="R2" s="19" t="n"/>
-      <c r="S2" s="19" t="n"/>
-      <c r="T2" s="19" t="n"/>
-      <c r="U2" s="19" t="n"/>
-      <c r="V2" s="19" t="n"/>
-      <c r="W2" s="19" t="n"/>
-      <c r="X2" s="19" t="n"/>
+      <c r="K2" s="28" t="n"/>
+      <c r="L2" s="28" t="n"/>
+      <c r="M2" s="28" t="n"/>
+      <c r="N2" s="28" t="n"/>
+      <c r="O2" s="28" t="n"/>
+      <c r="P2" s="28" t="n"/>
+      <c r="Q2" s="28" t="n"/>
+      <c r="R2" s="28" t="n"/>
+      <c r="S2" s="28" t="n"/>
+      <c r="T2" s="28" t="n"/>
+      <c r="U2" s="28" t="n"/>
+      <c r="V2" s="28" t="n"/>
+      <c r="W2" s="28" t="n"/>
+      <c r="X2" s="28" t="n"/>
+      <c r="Y2" s="28" t="n"/>
+      <c r="Z2" s="28" t="n"/>
+      <c r="AA2" s="28" t="n"/>
+      <c r="AB2" s="28" t="n"/>
+      <c r="AC2" s="28" t="n"/>
+      <c r="AD2" s="28" t="n"/>
+      <c r="AE2" s="28" t="n"/>
+      <c r="AF2" s="28" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="29" t="inlineStr">
         <is>
           <t>TVAE</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="30" t="n">
         <v>650</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="30" t="n">
         <v>200</v>
       </c>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n">
+      <c r="D3" s="30" t="n"/>
+      <c r="E3" s="30" t="n"/>
+      <c r="F3" s="30" t="n"/>
+      <c r="G3" s="30" t="n"/>
+      <c r="H3" s="30" t="n"/>
+      <c r="I3" s="30" t="n"/>
+      <c r="J3" s="30" t="n"/>
+      <c r="K3" s="30" t="n">
         <v>64</v>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>[128, 128]</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="30" t="inlineStr">
         <is>
           <t>[256, 256]</t>
         </is>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="N3" s="30" t="n">
         <v>0.0005284384205738843</v>
       </c>
-      <c r="O3" s="4" t="n">
+      <c r="O3" s="30" t="n">
         <v>10</v>
       </c>
-      <c r="P3" s="4" t="n"/>
-      <c r="Q3" s="4" t="n"/>
-      <c r="R3" s="4" t="n"/>
-      <c r="S3" s="4" t="n"/>
-      <c r="T3" s="4" t="n"/>
-      <c r="U3" s="4" t="n"/>
-      <c r="V3" s="4" t="n"/>
-      <c r="W3" s="4" t="n"/>
-      <c r="X3" s="4" t="n"/>
+      <c r="P3" s="30" t="n"/>
+      <c r="Q3" s="30" t="n"/>
+      <c r="R3" s="30" t="n"/>
+      <c r="S3" s="30" t="n"/>
+      <c r="T3" s="30" t="n"/>
+      <c r="U3" s="30" t="n"/>
+      <c r="V3" s="30" t="n"/>
+      <c r="W3" s="30" t="n"/>
+      <c r="X3" s="30" t="n"/>
+      <c r="Y3" s="30" t="n"/>
+      <c r="Z3" s="30" t="n"/>
+      <c r="AA3" s="30" t="n"/>
+      <c r="AB3" s="30" t="n"/>
+      <c r="AC3" s="30" t="n"/>
+      <c r="AD3" s="30" t="n"/>
+      <c r="AE3" s="30" t="n"/>
+      <c r="AF3" s="30" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>CTGAN</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="30" t="n">
         <v>1000</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="30" t="n">
         <v>200</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="30" t="n">
         <v>5.463331403485189e-05</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="30" t="n">
         <v>0.0001440313010173896</v>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="30" t="inlineStr">
         <is>
           <t>[256, 256, 256]</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="30" t="inlineStr">
         <is>
           <t>[512, 512]</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
-      <c r="O4" s="4" t="n"/>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="4" t="n"/>
-      <c r="R4" s="4" t="n"/>
-      <c r="S4" s="4" t="n"/>
-      <c r="T4" s="4" t="n"/>
-      <c r="U4" s="4" t="n"/>
-      <c r="V4" s="4" t="n"/>
-      <c r="W4" s="4" t="n"/>
-      <c r="X4" s="4" t="n"/>
+      <c r="J4" s="30" t="n"/>
+      <c r="K4" s="30" t="n"/>
+      <c r="L4" s="30" t="n"/>
+      <c r="M4" s="30" t="n"/>
+      <c r="N4" s="30" t="n"/>
+      <c r="O4" s="30" t="n"/>
+      <c r="P4" s="30" t="n"/>
+      <c r="Q4" s="30" t="n"/>
+      <c r="R4" s="30" t="n"/>
+      <c r="S4" s="30" t="n"/>
+      <c r="T4" s="30" t="n"/>
+      <c r="U4" s="30" t="n"/>
+      <c r="V4" s="30" t="n"/>
+      <c r="W4" s="30" t="n"/>
+      <c r="X4" s="30" t="n"/>
+      <c r="Y4" s="30" t="n"/>
+      <c r="Z4" s="30" t="n"/>
+      <c r="AA4" s="30" t="n"/>
+      <c r="AB4" s="30" t="n"/>
+      <c r="AC4" s="30" t="n"/>
+      <c r="AD4" s="30" t="n"/>
+      <c r="AE4" s="30" t="n"/>
+      <c r="AF4" s="30" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>GaussianCopula</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="B5" s="30" t="n"/>
+      <c r="C5" s="30" t="n"/>
+      <c r="D5" s="30" t="n"/>
+      <c r="E5" s="30" t="n"/>
+      <c r="F5" s="30" t="n"/>
+      <c r="G5" s="30" t="n"/>
+      <c r="H5" s="30" t="n"/>
+      <c r="I5" s="30" t="n"/>
+      <c r="J5" s="30" t="inlineStr">
         <is>
           <t>gamma</t>
         </is>
       </c>
-      <c r="K5" s="4" t="n"/>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="n"/>
-      <c r="N5" s="4" t="n"/>
-      <c r="O5" s="4" t="n"/>
-      <c r="P5" s="4" t="b">
+      <c r="K5" s="30" t="n"/>
+      <c r="L5" s="30" t="n"/>
+      <c r="M5" s="30" t="n"/>
+      <c r="N5" s="30" t="n"/>
+      <c r="O5" s="30" t="n"/>
+      <c r="P5" s="30" t="b">
         <v>1</v>
       </c>
-      <c r="Q5" s="4" t="n"/>
-      <c r="R5" s="4" t="n"/>
-      <c r="S5" s="4" t="n"/>
-      <c r="T5" s="4" t="n"/>
-      <c r="U5" s="4" t="n"/>
-      <c r="V5" s="4" t="n"/>
-      <c r="W5" s="4" t="n"/>
-      <c r="X5" s="4" t="n"/>
+      <c r="Q5" s="30" t="n"/>
+      <c r="R5" s="30" t="n"/>
+      <c r="S5" s="30" t="n"/>
+      <c r="T5" s="30" t="n"/>
+      <c r="U5" s="30" t="n"/>
+      <c r="V5" s="30" t="n"/>
+      <c r="W5" s="30" t="n"/>
+      <c r="X5" s="30" t="n"/>
+      <c r="Y5" s="30" t="n"/>
+      <c r="Z5" s="30" t="n"/>
+      <c r="AA5" s="30" t="n"/>
+      <c r="AB5" s="30" t="n"/>
+      <c r="AC5" s="30" t="n"/>
+      <c r="AD5" s="30" t="n"/>
+      <c r="AE5" s="30" t="n"/>
+      <c r="AF5" s="30" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>WGAN-GP</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="30" t="n">
         <v>1700</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="30" t="n">
         <v>128</v>
       </c>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="4" t="n"/>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="4" t="n"/>
-      <c r="K6" s="4" t="n"/>
-      <c r="L6" s="4" t="n"/>
-      <c r="M6" s="4" t="n"/>
-      <c r="N6" s="4" t="n"/>
-      <c r="O6" s="4" t="n"/>
-      <c r="P6" s="4" t="n"/>
-      <c r="Q6" s="4" t="n">
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="30" t="n"/>
+      <c r="F6" s="30" t="n"/>
+      <c r="G6" s="30" t="n"/>
+      <c r="H6" s="30" t="n"/>
+      <c r="I6" s="30" t="n"/>
+      <c r="J6" s="30" t="n"/>
+      <c r="K6" s="30" t="n"/>
+      <c r="L6" s="30" t="n"/>
+      <c r="M6" s="30" t="n"/>
+      <c r="N6" s="30" t="n"/>
+      <c r="O6" s="30" t="n"/>
+      <c r="P6" s="30" t="n"/>
+      <c r="Q6" s="30" t="n">
         <v>32</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="R6" s="30" t="n">
         <v>256</v>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="S6" s="30" t="n">
         <v>0.0001146615805893371</v>
       </c>
-      <c r="T6" s="4" t="n">
+      <c r="T6" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="U6" s="4" t="n">
+      <c r="U6" s="30" t="n">
         <v>1.589465151982894</v>
       </c>
-      <c r="V6" s="4" t="n"/>
-      <c r="W6" s="4" t="n"/>
-      <c r="X6" s="4" t="n"/>
+      <c r="V6" s="30" t="n"/>
+      <c r="W6" s="30" t="n"/>
+      <c r="X6" s="30" t="n"/>
+      <c r="Y6" s="30" t="n"/>
+      <c r="Z6" s="30" t="n"/>
+      <c r="AA6" s="30" t="n"/>
+      <c r="AB6" s="30" t="n"/>
+      <c r="AC6" s="30" t="n"/>
+      <c r="AD6" s="30" t="n"/>
+      <c r="AE6" s="30" t="n"/>
+      <c r="AF6" s="30" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>CTAB-GAN+</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="30" t="n">
         <v>275</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="30" t="n">
         <v>500</v>
       </c>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="4" t="n"/>
-      <c r="I7" s="4" t="n"/>
-      <c r="J7" s="4" t="n"/>
-      <c r="K7" s="4" t="n"/>
-      <c r="L7" s="4" t="n"/>
-      <c r="M7" s="4" t="n"/>
-      <c r="N7" s="4" t="n">
+      <c r="D7" s="30" t="n"/>
+      <c r="E7" s="30" t="n"/>
+      <c r="F7" s="30" t="n"/>
+      <c r="G7" s="30" t="n"/>
+      <c r="H7" s="30" t="n"/>
+      <c r="I7" s="30" t="n"/>
+      <c r="J7" s="30" t="n"/>
+      <c r="K7" s="30" t="n"/>
+      <c r="L7" s="30" t="n"/>
+      <c r="M7" s="30" t="n"/>
+      <c r="N7" s="30" t="n">
         <v>5.113822416024185e-05</v>
       </c>
-      <c r="O7" s="4" t="n"/>
-      <c r="P7" s="4" t="n"/>
-      <c r="Q7" s="4" t="n"/>
-      <c r="R7" s="4" t="n"/>
-      <c r="S7" s="4" t="n"/>
-      <c r="T7" s="4" t="n"/>
-      <c r="U7" s="4" t="n"/>
-      <c r="V7" s="4" t="n">
+      <c r="O7" s="30" t="n"/>
+      <c r="P7" s="30" t="n"/>
+      <c r="Q7" s="30" t="n"/>
+      <c r="R7" s="30" t="n"/>
+      <c r="S7" s="30" t="n"/>
+      <c r="T7" s="30" t="n"/>
+      <c r="U7" s="30" t="n"/>
+      <c r="V7" s="30" t="n">
         <v>100</v>
       </c>
-      <c r="W7" s="4" t="n">
+      <c r="W7" s="30" t="n">
         <v>128</v>
       </c>
-      <c r="X7" s="4" t="inlineStr">
+      <c r="X7" s="30" t="inlineStr">
         <is>
           <t>[128, 128, 128]</t>
+        </is>
+      </c>
+      <c r="Y7" s="30" t="n"/>
+      <c r="Z7" s="30" t="n"/>
+      <c r="AA7" s="30" t="n"/>
+      <c r="AB7" s="30" t="n"/>
+      <c r="AC7" s="30" t="n"/>
+      <c r="AD7" s="30" t="n"/>
+      <c r="AE7" s="30" t="n"/>
+      <c r="AF7" s="30" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>TabDDPM</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="n"/>
+      <c r="C8" s="30" t="n">
+        <v>256</v>
+      </c>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="30" t="n"/>
+      <c r="F8" s="30" t="n"/>
+      <c r="G8" s="30" t="n"/>
+      <c r="H8" s="30" t="n"/>
+      <c r="I8" s="30" t="n"/>
+      <c r="J8" s="30" t="n"/>
+      <c r="K8" s="30" t="n"/>
+      <c r="L8" s="30" t="n"/>
+      <c r="M8" s="30" t="n"/>
+      <c r="N8" s="30" t="n"/>
+      <c r="O8" s="30" t="n"/>
+      <c r="P8" s="30" t="n"/>
+      <c r="Q8" s="30" t="n"/>
+      <c r="R8" s="30" t="n"/>
+      <c r="S8" s="30" t="n">
+        <v>8.468008575248323e-05</v>
+      </c>
+      <c r="T8" s="30" t="n"/>
+      <c r="U8" s="30" t="n"/>
+      <c r="V8" s="30" t="n"/>
+      <c r="W8" s="30" t="n"/>
+      <c r="X8" s="30" t="n"/>
+      <c r="Y8" s="30" t="n">
+        <v>100</v>
+      </c>
+      <c r="Z8" s="30" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AA8" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB8" s="30" t="n">
+        <v>128</v>
+      </c>
+      <c r="AC8" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD8" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="30" t="inlineStr">
+        <is>
+          <t>cosine</t>
+        </is>
+      </c>
+      <c r="AF8" s="30" t="inlineStr">
+        <is>
+          <t>mse</t>
         </is>
       </c>
     </row>

</xml_diff>